<commit_message>
adding noew coptic font
</commit_message>
<xml_diff>
--- a/exams_import.xlsx
+++ b/exams_import.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\MY_WORK\peter\qr-exams-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E627841-D79E-432A-9439-00245335C4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96510547-23EA-4CBA-9C3C-2D4C0CCA1E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="2268" windowWidth="17280" windowHeight="8964" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="22">
   <si>
     <t>type</t>
   </si>
@@ -1087,4 +1088,289 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEAA58B4-CCC6-449D-B1B2-34A66B80EAA5}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>